<commit_message>
Receiver Server Capability - Bundle Transaction support  [FHIR-51401](https://jira.hl7.org/browse/FHIR-51401). Also updated Receiver Server and Reporter Client spreadsheets. Also updated change-notes and package_list.yml Also corrected summary component weighted MeasureReport example.
</commit_message>
<xml_diff>
--- a/input/resources/source-data/DEQM_Capability_Statement_Receiver_Server.xlsx
+++ b/input/resources/source-data/DEQM_Capability_Statement_Receiver_Server.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\davinci-deqm\input\resources\source-data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SourceControl\Git\HL7\davinci-deqm\input\resources\source-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2992D826-350F-4AAA-82D2-84558B7E6B2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FCF5F03-081B-4A08-A555-DFD94FADD6C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3312" yWindow="1020" windowWidth="26052" windowHeight="15240" activeTab="3" xr2:uid="{33C1B24A-521B-4A24-AA1F-999D8048322A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="7" xr2:uid="{33C1B24A-521B-4A24-AA1F-999D8048322A}"/>
   </bookViews>
   <sheets>
     <sheet name="config" sheetId="11" r:id="rId1"/>
@@ -27,7 +27,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">profiles!$A$1:$D$11</definedName>
   </definedNames>
-  <calcPr calcId="191029" refMode="R1C1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -487,6 +487,27 @@
     <t>!http://hl7.org/fhir/us/davinci-deqm/StructureDefinition/devicerequest-deqm</t>
   </si>
   <si>
+    <t>http://hl7.org/fhir/us/davinci-deqm/</t>
+  </si>
+  <si>
+    <t>3.1.0</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/us/davinci-deqm/ImplementationGuide/hl7.fhir.us.davinci-deqm|3.1.0</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/us/qicore/ImplementationGuide/hl7.fhir.us.qicore|4.1.1</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/us/cqfmeasures/ImplementationGuide/hl7.fhir.us.cqfmeasures|3.0.0</t>
+  </si>
+  <si>
+    <t>!http://hl7.org/fhir/us/qicore/StructureDefinition/qicore-organization</t>
+  </si>
+  <si>
+    <t>QI Core Organization Profile</t>
+  </si>
+  <si>
     <t xml:space="preserve">Da Vinci DEQM Producer Server **SHALL**
 1. Support the following  transactions defined in the *Framework* Section of  this  Implementation Guide:
    - Individual Reporting
@@ -494,28 +515,8 @@
 1. Declare a CapabilityStatement identifying the list of supported profiles and operations.
 1. Implement the FHIR RESTful API for operations including returning the appropriate response classes as described in the FHIR specification for [Extended Operations on the RESTful API ](http://hl7.org/fhir/R4/operations.html).
 1. Support both xml and json resource formats for all interactions.
+1. Support support for one of 'batch' or 'transaction'.
 </t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/us/davinci-deqm/</t>
-  </si>
-  <si>
-    <t>3.1.0</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/us/davinci-deqm/ImplementationGuide/hl7.fhir.us.davinci-deqm|3.1.0</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/us/qicore/ImplementationGuide/hl7.fhir.us.qicore|4.1.1</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/us/cqfmeasures/ImplementationGuide/hl7.fhir.us.cqfmeasures|3.0.0</t>
-  </si>
-  <si>
-    <t>!http://hl7.org/fhir/us/qicore/StructureDefinition/qicore-organization</t>
-  </si>
-  <si>
-    <t>QI Core Organization Profile</t>
   </si>
 </sst>
 </file>
@@ -603,7 +604,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -612,7 +613,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFill="1"/>
@@ -636,9 +636,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -676,7 +676,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -782,7 +782,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -924,7 +924,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -933,9 +933,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB9BF198-9F92-4812-A64F-4AD3FCDA511C}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>44</v>
       </c>
@@ -943,7 +943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>115</v>
       </c>
@@ -951,7 +951,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>117</v>
       </c>
@@ -959,7 +959,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>119</v>
       </c>
@@ -967,15 +967,15 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>121</v>
       </c>
       <c r="B5" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>122</v>
       </c>
@@ -983,7 +983,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>124</v>
       </c>
@@ -991,7 +991,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>126</v>
       </c>
@@ -1007,21 +1007,21 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7399C2ED-EDEB-47AB-8C1E-1290512B1D2F}">
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="63.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.6640625" customWidth="1"/>
-    <col min="3" max="3" width="19.44140625" customWidth="1"/>
-    <col min="4" max="5" width="9.109375" customWidth="1"/>
-    <col min="6" max="6" width="22.6640625" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" customWidth="1"/>
-    <col min="8" max="8" width="34.6640625" customWidth="1"/>
-    <col min="9" max="15" width="9.109375" customWidth="1"/>
-    <col min="16" max="16" width="14.44140625" customWidth="1"/>
-    <col min="17" max="17" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="63.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" customWidth="1"/>
+    <col min="4" max="5" width="9.140625" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" customWidth="1"/>
+    <col min="8" max="8" width="34.7109375" customWidth="1"/>
+    <col min="9" max="15" width="9.140625" customWidth="1"/>
+    <col min="16" max="16" width="14.42578125" customWidth="1"/>
+    <col min="17" max="17" width="20.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -1074,7 +1074,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
     </row>
   </sheetData>
@@ -1085,13 +1085,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A15F3286-55C1-40D0-93FC-C97EF26956B8}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.6640625" customWidth="1"/>
-    <col min="2" max="2" width="95.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.7109375" customWidth="1"/>
+    <col min="2" max="2" width="95.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1099,15 +1099,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>75</v>
       </c>
       <c r="B2" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>76</v>
       </c>
@@ -1115,7 +1115,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1123,7 +1123,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1131,15 +1131,15 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B6" s="6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1147,15 +1147,15 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="172.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -1174,12 +1174,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0829A918-BBB6-6345-897C-371FBE4213DF}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="68.33203125" customWidth="1"/>
+    <col min="2" max="2" width="68.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>45</v>
       </c>
@@ -1187,20 +1187,20 @@
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>140</v>
+      <c r="B3" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -1211,15 +1211,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B139EF60-0633-48C5-B394-C56F006BD6B3}">
   <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="98.44140625" customWidth="1"/>
-    <col min="2" max="2" width="60.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.109375" customWidth="1"/>
-    <col min="4" max="4" width="16.109375" customWidth="1"/>
+    <col min="1" max="1" width="98.42578125" customWidth="1"/>
+    <col min="2" max="2" width="60.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.140625" customWidth="1"/>
+    <col min="4" max="4" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -1233,7 +1233,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>134</v>
       </c>
@@ -1247,7 +1247,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>133</v>
       </c>
@@ -1261,7 +1261,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>112</v>
       </c>
@@ -1275,7 +1275,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>132</v>
       </c>
@@ -1289,7 +1289,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>131</v>
       </c>
@@ -1303,12 +1303,12 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B7" t="s">
         <v>141</v>
-      </c>
-      <c r="B7" t="s">
-        <v>142</v>
       </c>
       <c r="C7" t="s">
         <v>5</v>
@@ -1317,7 +1317,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>130</v>
       </c>
@@ -1331,7 +1331,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>113</v>
       </c>
@@ -1345,7 +1345,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>129</v>
       </c>
@@ -1359,7 +1359,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>114</v>
       </c>
@@ -1383,19 +1383,19 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0ACB4CFA-AAEF-4FC6-A49B-107CEE80A317}">
   <dimension ref="A1:X3"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="36.44140625" customWidth="1"/>
-    <col min="2" max="2" width="25.33203125" customWidth="1"/>
+    <col min="1" max="1" width="36.42578125" customWidth="1"/>
+    <col min="2" max="2" width="25.28515625" customWidth="1"/>
     <col min="3" max="3" width="53" customWidth="1"/>
-    <col min="4" max="4" width="15.109375" customWidth="1"/>
-    <col min="5" max="6" width="17.44140625" customWidth="1"/>
-    <col min="7" max="7" width="20.44140625" customWidth="1"/>
-    <col min="8" max="8" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.44140625" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" customWidth="1"/>
+    <col min="5" max="6" width="17.42578125" customWidth="1"/>
+    <col min="7" max="7" width="20.42578125" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:24" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>39</v>
       </c>
@@ -1453,23 +1453,23 @@
       <c r="S1" t="s">
         <v>88</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="T1" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="U1" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="V1" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="W1" s="5" t="s">
+      <c r="W1" s="4" t="s">
         <v>92</v>
       </c>
       <c r="X1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:24" ht="58.2" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" ht="60.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>52</v>
       </c>
@@ -1480,7 +1480,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C3" s="2"/>
     </row>
   </sheetData>
@@ -1496,14 +1496,14 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="59" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.109375" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>45</v>
       </c>
@@ -1529,15 +1529,15 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9E2E280-092F-4777-8984-8212A8DAB750}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-    <col min="2" max="2" width="24.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.44140625" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>41</v>
       </c>
@@ -1545,7 +1545,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>29</v>
       </c>
@@ -1553,22 +1553,22 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>33</v>
       </c>
@@ -1576,12 +1576,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>35</v>
       </c>
@@ -1589,12 +1589,12 @@
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>37</v>
       </c>
@@ -1607,13 +1607,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F751A03-03CC-424E-A8A3-C2D24B8653CA}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.109375" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>41</v>
       </c>
@@ -1624,16 +1624,16 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>94</v>
       </c>
       <c r="B2" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>96</v>
       </c>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>97</v>
       </c>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="C4" s="1"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>98</v>
       </c>
@@ -1668,41 +1668,41 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBB2A2CB-11AF-4645-811D-C66964301C49}">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" ht="18" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="4" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1722,7 +1722,7 @@
       <c r="F2" t="s">
         <v>111</v>
       </c>
-      <c r="J2" s="6" t="str">
+      <c r="J2" s="5" t="str">
         <f t="shared" ref="J2" si="1">"Fetches a bundle of all "&amp;B2&amp;" resources matching the specified "&amp;SUBSTITUTE(D2,","," and ")</f>
         <v>Fetches a bundle of all !Encounter resources matching the specified class and date</v>
       </c>

</xml_diff>